<commit_message>
use Okabe–Ito colorblind-safe palette
</commit_message>
<xml_diff>
--- a/ProteomeXChange/false_classification_review_v1.xlsx
+++ b/ProteomeXChange/false_classification_review_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/owensun/Downloads/code/finding-datasets-with-LLMs/ProteomeXChange/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0E2885E-3968-9A4C-85A1-F7B8CF6BD17D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EFE9EBE-9DB0-8B49-B05F-E1B210861949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_root_causes" sheetId="1" state="hidden" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="144">
   <si>
     <t>dataset_id</t>
   </si>
@@ -443,14 +443,33 @@
     <t>Misinterpreted: if there is no healthy controls proportion noted, include it — for additional human review.</t>
   </si>
   <si>
-    <t>Clarification: healthy or non-malignant patient controls.</t>
+    <t>Healthy tissue is from healthy regions of serous ovarian cancers. Intended is healthy tissue from healthy patients.</t>
+  </si>
+  <si>
+    <t>Healthy tissue is from healthy regions of serous ovarian cancers. Intended is healthy tissue from healthy patients.
+"disease-free omentum from patient with non-metastatic ovarian cancer and high-grade- serous-ovarian- cancer-derived omental metastasis samples"</t>
+  </si>
+  <si>
+    <t>Benign tumors vs. metastatic. Intended is healthy tissue from healthy patients.</t>
+  </si>
+  <si>
+    <t>Not about ovarian cancer.</t>
+  </si>
+  <si>
+    <t>Xenograft study.</t>
+  </si>
+  <si>
+    <t>Ex vivo study.</t>
+  </si>
+  <si>
+    <t>Clarificiation: diagnostic biomarker discovery studies should be included as the target meta-analysis is about diagnostic biomarker discovery.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -505,7 +524,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -516,25 +535,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDDEBF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="20">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -974,64 +982,64 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1">
       <c r="A5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:1">
       <c r="A6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1">
       <c r="A7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:1">
       <c r="A8" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:1">
       <c r="A9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:1">
       <c r="A10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:1">
       <c r="A11" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:1">
       <c r="A12" t="s">
         <v>56</v>
       </c>
@@ -1044,7 +1052,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -1058,7 +1066,7 @@
     <col min="16" max="16" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="16">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1108,7 +1116,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="64">
       <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
@@ -1156,7 +1164,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="80">
       <c r="A3" s="3" t="s">
         <v>28</v>
       </c>
@@ -1204,7 +1212,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="80">
       <c r="A4" s="3" t="s">
         <v>34</v>
       </c>
@@ -1248,11 +1256,11 @@
         <v>27</v>
       </c>
       <c r="O4" s="3"/>
-      <c r="P4" s="3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+      <c r="P4" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="80">
       <c r="A5" s="3" t="s">
         <v>40</v>
       </c>
@@ -1303,10 +1311,10 @@
   </sheetData>
   <autoFilter ref="A1:P5" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <conditionalFormatting sqref="A2:P3 A5:P5 A4:O4">
-    <cfRule type="expression" dxfId="21" priority="3">
+    <cfRule type="expression" dxfId="19" priority="3">
       <formula>$H2="FP"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="4">
+    <cfRule type="expression" dxfId="18" priority="4">
       <formula>$H2="FN"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1338,7 +1346,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -1352,7 +1360,7 @@
     <col min="16" max="16" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="16">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1402,405 +1410,418 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:16" ht="64">
+      <c r="A2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="3" t="b">
+      <c r="F2" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G2" s="3" t="b">
+      <c r="G2" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-    </row>
-    <row r="3" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="O2" s="4"/>
+      <c r="P2" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="112">
+      <c r="A3" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="3" t="b">
+      <c r="F3" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G3" s="3" t="b">
+      <c r="G3" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-    </row>
-    <row r="4" spans="1:16" ht="80" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="O3" s="4"/>
+      <c r="P3" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="80">
+      <c r="A4" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="3" t="b">
+      <c r="F4" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G4" s="3" t="b">
+      <c r="G4" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-    </row>
-    <row r="5" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="O4" s="4"/>
+      <c r="P4" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="64">
+      <c r="A5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="3" t="b">
+      <c r="F5" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="G5" s="3" t="b">
+      <c r="G5" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L5" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3" t="s">
+      <c r="O5" s="4"/>
+      <c r="P5" s="4" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:16" ht="64">
+      <c r="A6" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="3" t="b">
+      <c r="F6" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G6" s="3" t="b">
+      <c r="G6" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L6" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="M6" s="3" t="s">
+      <c r="M6" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="N6" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-    </row>
-    <row r="7" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="O6" s="4"/>
+      <c r="P6" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="64">
+      <c r="A7" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="3" t="b">
+      <c r="F7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G7" s="3" t="b">
+      <c r="G7" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="L7" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="M7" s="3" t="s">
+      <c r="M7" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="N7" s="3" t="s">
+      <c r="N7" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-    </row>
-    <row r="8" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+      <c r="O7" s="4"/>
+      <c r="P7" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="64">
+      <c r="A8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="3" t="b">
+      <c r="F8" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="G8" s="3" t="b">
+      <c r="G8" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="K8" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="L8" s="3" t="s">
+      <c r="L8" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="M8" s="3" t="s">
+      <c r="M8" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="N8" s="3" t="s">
+      <c r="N8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="96" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="O8" s="4"/>
+      <c r="P8" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="96">
+      <c r="A9" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="3" t="b">
+      <c r="F9" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G9" s="3" t="b">
+      <c r="G9" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="J9" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="K9" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="L9" s="3" t="s">
+      <c r="L9" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="M9" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="N9" s="3" t="s">
+      <c r="N9" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4" t="s">
+        <v>142</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:P9" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="A6:P7 A5:O5 A9:P9 A8:O8 A2:P4">
-    <cfRule type="expression" dxfId="19" priority="5">
+  <conditionalFormatting sqref="A4:P9 A2:O3">
+    <cfRule type="expression" dxfId="17" priority="5">
       <formula>$H2="FP"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="6">
+    <cfRule type="expression" dxfId="16" priority="6">
       <formula>$H2="FN"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P5">
-    <cfRule type="expression" dxfId="11" priority="3">
-      <formula>$H5="FP"</formula>
+  <conditionalFormatting sqref="P3">
+    <cfRule type="expression" dxfId="9" priority="3">
+      <formula>$H3="FP"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="4">
-      <formula>$H5="FN"</formula>
+    <cfRule type="expression" dxfId="8" priority="4">
+      <formula>$H3="FN"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P8">
-    <cfRule type="expression" dxfId="9" priority="1">
-      <formula>$H8="FP"</formula>
+  <conditionalFormatting sqref="P2">
+    <cfRule type="expression" dxfId="7" priority="1">
+      <formula>$H2="FP"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="2">
-      <formula>$H8="FN"</formula>
+    <cfRule type="expression" dxfId="6" priority="2">
+      <formula>$H2="FN"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
@@ -1819,7 +1840,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:P4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -1833,7 +1854,7 @@
     <col min="16" max="16" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="16">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1883,153 +1904,165 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="112" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:16" ht="112">
+      <c r="A2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="3" t="b">
+      <c r="F2" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G2" s="3" t="b">
+      <c r="G2" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-    </row>
-    <row r="3" spans="1:16" ht="112" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="O2" s="4"/>
+      <c r="P2" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="112">
+      <c r="A3" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="3" t="b">
+      <c r="F3" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G3" s="3" t="b">
+      <c r="G3" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-    </row>
-    <row r="4" spans="1:16" ht="96" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="O3" s="4"/>
+      <c r="P3" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="96">
+      <c r="A4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="3" t="b">
+      <c r="F4" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="G4" s="3" t="b">
+      <c r="G4" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3" t="s">
-        <v>137</v>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:P4" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="A2:P3 A4:O4">
-    <cfRule type="expression" dxfId="17" priority="5">
+  <conditionalFormatting sqref="A2:O4">
+    <cfRule type="expression" dxfId="15" priority="5">
       <formula>$H2="FP"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="6">
+    <cfRule type="expression" dxfId="14" priority="6">
+      <formula>$H2="FN"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P2:P3">
+    <cfRule type="expression" dxfId="11" priority="3">
+      <formula>$H2="FP"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="4">
       <formula>$H2="FN"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2060,7 +2093,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:P3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -2074,7 +2107,7 @@
     <col min="16" max="16" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="16">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2124,107 +2157,109 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:16" ht="64">
+      <c r="A2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="3" t="b">
+      <c r="F2" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G2" s="3" t="b">
+      <c r="G2" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-    </row>
-    <row r="3" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="O2" s="4"/>
+      <c r="P2" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="64">
+      <c r="A3" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="3" t="b">
+      <c r="F3" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="G3" s="3" t="b">
+      <c r="G3" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3" t="s">
-        <v>137</v>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:P3" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <conditionalFormatting sqref="A2:P2 A3:O3">
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="13" priority="3">
       <formula>$H2="FP"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="12" priority="4">
       <formula>$H2="FN"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2237,6 +2272,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">

</xml_diff>